<commit_message>
feat(page-auto): update posting workflow
</commit_message>
<xml_diff>
--- a/data/databook.xlsx
+++ b/data/databook.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="684">
   <si>
     <t>profile_id</t>
   </si>
@@ -158,10 +158,7 @@
     <t>PAGE-001</t>
   </si>
   <si>
-    <t>Test 1</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/profile.php?id=61595080421933</t>
+    <t>PAUSED</t>
   </si>
   <si>
     <t>PAGE-002</t>
@@ -319,17 +316,36 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <color rgb="FF800080"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">FULL STORY IN HERE ❤👇👇:
+      <t xml:space="preserve">FULL STORY IN HERE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF800080"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>❤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF800080"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">👇👇:
 </t>
     </r>
     <r>
       <rPr>
         <u/>
         <sz val="10"/>
-        <color rgb="FF1155CC"/>
+        <color rgb="FF800080"/>
         <rFont val="宋体"/>
         <charset val="134"/>
       </rPr>
@@ -14971,7 +14987,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="31">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -14993,6 +15009,12 @@
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -15167,6 +15189,19 @@
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF800080"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -15542,31 +15577,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -15575,115 +15607,118 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -15707,20 +15742,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="6" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="6" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16523,31 +16558,25 @@
       <c r="A2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:5">
       <c r="A3" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>27</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>46</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>7</v>
@@ -16555,7 +16584,7 @@
     </row>
     <row r="4" customHeight="1" spans="1:5">
       <c r="A4" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -16564,7 +16593,7 @@
     </row>
     <row r="5" customHeight="1" spans="1:5">
       <c r="A5" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -16573,7 +16602,7 @@
     </row>
     <row r="6" customHeight="1" spans="1:5">
       <c r="A6" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -16582,7 +16611,7 @@
     </row>
     <row r="7" customHeight="1" spans="1:5">
       <c r="A7" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -16591,7 +16620,7 @@
     </row>
     <row r="8" customHeight="1" spans="1:5">
       <c r="A8" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -16600,7 +16629,7 @@
     </row>
     <row r="9" customHeight="1" spans="1:5">
       <c r="A9" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -16609,7 +16638,7 @@
     </row>
     <row r="10" customHeight="1" spans="1:5">
       <c r="A10" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -16618,7 +16647,7 @@
     </row>
     <row r="11" customHeight="1" spans="1:5">
       <c r="A11" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -16627,7 +16656,7 @@
     </row>
     <row r="12" customHeight="1" spans="1:5">
       <c r="A12" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -16636,7 +16665,7 @@
     </row>
     <row r="13" customHeight="1" spans="1:5">
       <c r="A13" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -16645,7 +16674,7 @@
     </row>
     <row r="14" customHeight="1" spans="1:5">
       <c r="A14" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -16654,7 +16683,7 @@
     </row>
     <row r="15" customHeight="1" spans="1:5">
       <c r="A15" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -16663,7 +16692,7 @@
     </row>
     <row r="16" customHeight="1" spans="1:5">
       <c r="A16" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -16672,7 +16701,7 @@
     </row>
     <row r="17" customHeight="1" spans="1:5">
       <c r="A17" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -16681,7 +16710,7 @@
     </row>
     <row r="18" customHeight="1" spans="1:5">
       <c r="A18" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -16690,7 +16719,7 @@
     </row>
     <row r="19" customHeight="1" spans="1:5">
       <c r="A19" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -16699,7 +16728,7 @@
     </row>
     <row r="20" customHeight="1" spans="1:5">
       <c r="A20" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -16708,7 +16737,7 @@
     </row>
     <row r="21" customHeight="1" spans="1:5">
       <c r="A21" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
@@ -16722,8 +16751,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="https://www.facebook.com/profile.php?id=61595080421933"/>
-    <hyperlink ref="D3" r:id="rId2" display="https://www.facebook.com/profile.php?id=61594947346869"/>
+    <hyperlink ref="D3" r:id="rId1" display="https://www.facebook.com/profile.php?id=61594947346869"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -16745,42 +16773,38 @@
   <sheetData>
     <row r="1" ht="12.75" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:26">
       <c r="A2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
@@ -16805,22 +16829,22 @@
     </row>
     <row r="3" customHeight="1" spans="1:26">
       <c r="A3" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -16845,22 +16869,18 @@
     </row>
     <row r="4" customHeight="1" spans="1:26">
       <c r="A4" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>81</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -16885,22 +16905,22 @@
     </row>
     <row r="5" customHeight="1" spans="1:26">
       <c r="A5" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="5">
         <v>2</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -16925,22 +16945,18 @@
     </row>
     <row r="6" customHeight="1" spans="1:26">
       <c r="A6" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="6">
-        <v>3</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -16965,22 +16981,22 @@
     </row>
     <row r="7" customHeight="1" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" s="2">
         <v>3</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -17005,22 +17021,18 @@
     </row>
     <row r="8" customHeight="1" spans="1:26">
       <c r="A8" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="5">
-        <v>4</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -17045,22 +17057,22 @@
     </row>
     <row r="9" customHeight="1" spans="1:26">
       <c r="A9" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" s="5">
         <v>4</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -17085,22 +17097,18 @@
     </row>
     <row r="10" customHeight="1" spans="1:26">
       <c r="A10" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="5">
-        <v>5</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -17125,22 +17133,22 @@
     </row>
     <row r="11" customHeight="1" spans="1:26">
       <c r="A11" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="6">
         <v>5</v>
       </c>
       <c r="D11" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>109</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -17165,18 +17173,18 @@
     </row>
     <row r="12" customHeight="1" spans="1:26">
       <c r="A12" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -17201,18 +17209,18 @@
     </row>
     <row r="13" customHeight="1" spans="1:26">
       <c r="A13" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>116</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>117</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -17237,18 +17245,18 @@
     </row>
     <row r="14" customHeight="1" spans="1:26">
       <c r="A14" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -17273,18 +17281,18 @@
     </row>
     <row r="15" customHeight="1" spans="1:26">
       <c r="A15" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -17309,18 +17317,18 @@
     </row>
     <row r="16" customHeight="1" spans="1:26">
       <c r="A16" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -17345,16 +17353,16 @@
     </row>
     <row r="17" customHeight="1" spans="1:26">
       <c r="A17" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -17379,16 +17387,16 @@
     </row>
     <row r="18" customHeight="1" spans="1:26">
       <c r="A18" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -17413,16 +17421,16 @@
     </row>
     <row r="19" customHeight="1" spans="1:26">
       <c r="A19" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -17447,16 +17455,16 @@
     </row>
     <row r="20" customHeight="1" spans="1:26">
       <c r="A20" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -17481,16 +17489,16 @@
     </row>
     <row r="21" customHeight="1" spans="1:26">
       <c r="A21" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -17515,16 +17523,16 @@
     </row>
     <row r="22" customHeight="1" spans="1:26">
       <c r="A22" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -17549,16 +17557,16 @@
     </row>
     <row r="23" customHeight="1" spans="1:26">
       <c r="A23" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E23" s="5"/>
       <c r="F23" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -17583,16 +17591,16 @@
     </row>
     <row r="24" customHeight="1" spans="1:26">
       <c r="A24" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -17617,16 +17625,16 @@
     </row>
     <row r="25" customHeight="1" spans="1:26">
       <c r="A25" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -17651,16 +17659,16 @@
     </row>
     <row r="26" customHeight="1" spans="1:26">
       <c r="A26" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -17685,16 +17693,16 @@
     </row>
     <row r="27" customHeight="1" spans="1:26">
       <c r="A27" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -17719,16 +17727,16 @@
     </row>
     <row r="28" customHeight="1" spans="1:26">
       <c r="A28" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -17753,16 +17761,16 @@
     </row>
     <row r="29" customHeight="1" spans="1:26">
       <c r="A29" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -17787,16 +17795,16 @@
     </row>
     <row r="30" customHeight="1" spans="1:26">
       <c r="A30" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
@@ -17821,16 +17829,16 @@
     </row>
     <row r="31" customHeight="1" spans="1:26">
       <c r="A31" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -17855,16 +17863,16 @@
     </row>
     <row r="32" customHeight="1" spans="1:26">
       <c r="A32" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -17889,16 +17897,16 @@
     </row>
     <row r="33" customHeight="1" spans="1:26">
       <c r="A33" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E33" s="5"/>
       <c r="F33" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -17923,16 +17931,16 @@
     </row>
     <row r="34" customHeight="1" spans="1:26">
       <c r="A34" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E34" s="5"/>
       <c r="F34" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
@@ -17957,16 +17965,16 @@
     </row>
     <row r="35" customHeight="1" spans="1:26">
       <c r="A35" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -17991,16 +17999,16 @@
     </row>
     <row r="36" customHeight="1" spans="1:26">
       <c r="A36" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -18025,16 +18033,16 @@
     </row>
     <row r="37" customHeight="1" spans="1:26">
       <c r="A37" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -18059,16 +18067,16 @@
     </row>
     <row r="38" customHeight="1" spans="1:26">
       <c r="A38" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E38" s="5"/>
       <c r="F38" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -18093,16 +18101,16 @@
     </row>
     <row r="39" customHeight="1" spans="1:26">
       <c r="A39" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E39" s="5"/>
       <c r="F39" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -18127,16 +18135,16 @@
     </row>
     <row r="40" customHeight="1" spans="1:26">
       <c r="A40" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -18161,16 +18169,16 @@
     </row>
     <row r="41" customHeight="1" spans="1:26">
       <c r="A41" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E41" s="6"/>
       <c r="F41" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -18195,16 +18203,16 @@
     </row>
     <row r="42" customHeight="1" spans="1:26">
       <c r="A42" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
@@ -18229,16 +18237,16 @@
     </row>
     <row r="43" customHeight="1" spans="1:26">
       <c r="A43" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E43" s="5"/>
       <c r="F43" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
@@ -18263,16 +18271,16 @@
     </row>
     <row r="44" customHeight="1" spans="1:26">
       <c r="A44" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -18297,16 +18305,16 @@
     </row>
     <row r="45" customHeight="1" spans="1:26">
       <c r="A45" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -18331,16 +18339,16 @@
     </row>
     <row r="46" customHeight="1" spans="1:26">
       <c r="A46" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E46" s="6"/>
       <c r="F46" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -18365,16 +18373,16 @@
     </row>
     <row r="47" customHeight="1" spans="1:26">
       <c r="A47" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -18399,16 +18407,16 @@
     </row>
     <row r="48" customHeight="1" spans="1:26">
       <c r="A48" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -18433,16 +18441,16 @@
     </row>
     <row r="49" customHeight="1" spans="1:26">
       <c r="A49" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -18467,16 +18475,16 @@
     </row>
     <row r="50" customHeight="1" spans="1:26">
       <c r="A50" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -18501,16 +18509,16 @@
     </row>
     <row r="51" customHeight="1" spans="1:26">
       <c r="A51" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
       <c r="D51" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E51" s="6"/>
       <c r="F51" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -18535,16 +18543,16 @@
     </row>
     <row r="52" customHeight="1" spans="1:26">
       <c r="A52" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -18569,16 +18577,16 @@
     </row>
     <row r="53" customHeight="1" spans="1:26">
       <c r="A53" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E53" s="5"/>
       <c r="F53" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -18603,16 +18611,16 @@
     </row>
     <row r="54" customHeight="1" spans="1:26">
       <c r="A54" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E54" s="5"/>
       <c r="F54" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -18637,16 +18645,16 @@
     </row>
     <row r="55" customHeight="1" spans="1:26">
       <c r="A55" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E55" s="5"/>
       <c r="F55" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -18671,16 +18679,16 @@
     </row>
     <row r="56" customHeight="1" spans="1:26">
       <c r="A56" s="6" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
       <c r="D56" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E56" s="6"/>
       <c r="F56" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -18705,16 +18713,16 @@
     </row>
     <row r="57" customHeight="1" spans="1:26">
       <c r="A57" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -18739,16 +18747,16 @@
     </row>
     <row r="58" customHeight="1" spans="1:26">
       <c r="A58" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -18773,16 +18781,16 @@
     </row>
     <row r="59" customHeight="1" spans="1:26">
       <c r="A59" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
       <c r="D59" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -18807,16 +18815,16 @@
     </row>
     <row r="60" customHeight="1" spans="1:26">
       <c r="A60" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
       <c r="D60" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -18841,16 +18849,16 @@
     </row>
     <row r="61" customHeight="1" spans="1:26">
       <c r="A61" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
       <c r="D61" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E61" s="6"/>
       <c r="F61" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -18875,16 +18883,16 @@
     </row>
     <row r="62" customHeight="1" spans="1:26">
       <c r="A62" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
@@ -18909,16 +18917,16 @@
     </row>
     <row r="63" customHeight="1" spans="1:26">
       <c r="A63" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B63" s="5"/>
       <c r="C63" s="5"/>
       <c r="D63" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -18943,16 +18951,16 @@
     </row>
     <row r="64" customHeight="1" spans="1:26">
       <c r="A64" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
       <c r="D64" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -18977,16 +18985,16 @@
     </row>
     <row r="65" customHeight="1" spans="1:26">
       <c r="A65" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B65" s="5"/>
       <c r="C65" s="5"/>
       <c r="D65" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -19011,16 +19019,16 @@
     </row>
     <row r="66" customHeight="1" spans="1:26">
       <c r="A66" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
       <c r="D66" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -19045,16 +19053,16 @@
     </row>
     <row r="67" customHeight="1" spans="1:26">
       <c r="A67" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E67" s="2"/>
       <c r="F67" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
@@ -19079,16 +19087,16 @@
     </row>
     <row r="68" customHeight="1" spans="1:26">
       <c r="A68" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
       <c r="D68" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -19113,16 +19121,16 @@
     </row>
     <row r="69" customHeight="1" spans="1:26">
       <c r="A69" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="5"/>
       <c r="D69" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -19147,16 +19155,16 @@
     </row>
     <row r="70" customHeight="1" spans="1:26">
       <c r="A70" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="5"/>
       <c r="D70" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -19181,16 +19189,16 @@
     </row>
     <row r="71" customHeight="1" spans="1:26">
       <c r="A71" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="6"/>
       <c r="D71" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -19215,16 +19223,16 @@
     </row>
     <row r="72" customHeight="1" spans="1:26">
       <c r="A72" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
@@ -19249,16 +19257,16 @@
     </row>
     <row r="73" customHeight="1" spans="1:26">
       <c r="A73" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
       <c r="D73" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E73" s="5"/>
       <c r="F73" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
@@ -19283,16 +19291,16 @@
     </row>
     <row r="74" customHeight="1" spans="1:26">
       <c r="A74" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
       <c r="D74" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E74" s="5"/>
       <c r="F74" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G74" s="4"/>
       <c r="H74" s="4"/>
@@ -19317,16 +19325,16 @@
     </row>
     <row r="75" customHeight="1" spans="1:26">
       <c r="A75" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
       <c r="D75" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E75" s="5"/>
       <c r="F75" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
@@ -19351,16 +19359,16 @@
     </row>
     <row r="76" customHeight="1" spans="1:26">
       <c r="A76" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
       <c r="D76" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E76" s="6"/>
       <c r="F76" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
@@ -19385,16 +19393,16 @@
     </row>
     <row r="77" customHeight="1" spans="1:26">
       <c r="A77" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E77" s="2"/>
       <c r="F77" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
@@ -19419,16 +19427,16 @@
     </row>
     <row r="78" customHeight="1" spans="1:26">
       <c r="A78" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
       <c r="D78" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E78" s="5"/>
       <c r="F78" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
@@ -19453,16 +19461,16 @@
     </row>
     <row r="79" customHeight="1" spans="1:26">
       <c r="A79" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B79" s="5"/>
       <c r="C79" s="5"/>
       <c r="D79" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E79" s="5"/>
       <c r="F79" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
@@ -19487,16 +19495,16 @@
     </row>
     <row r="80" customHeight="1" spans="1:26">
       <c r="A80" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B80" s="5"/>
       <c r="C80" s="5"/>
       <c r="D80" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E80" s="5"/>
       <c r="F80" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
@@ -19521,16 +19529,16 @@
     </row>
     <row r="81" customHeight="1" spans="1:26">
       <c r="A81" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B81" s="6"/>
       <c r="C81" s="6"/>
       <c r="D81" s="6" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E81" s="6"/>
       <c r="F81" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G81" s="4"/>
       <c r="H81" s="4"/>
@@ -19555,16 +19563,16 @@
     </row>
     <row r="82" customHeight="1" spans="1:26">
       <c r="A82" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E82" s="2"/>
       <c r="F82" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
@@ -19589,16 +19597,16 @@
     </row>
     <row r="83" customHeight="1" spans="1:26">
       <c r="A83" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B83" s="5"/>
       <c r="C83" s="5"/>
       <c r="D83" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E83" s="5"/>
       <c r="F83" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
@@ -19623,16 +19631,16 @@
     </row>
     <row r="84" customHeight="1" spans="1:26">
       <c r="A84" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B84" s="5"/>
       <c r="C84" s="5"/>
       <c r="D84" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E84" s="5"/>
       <c r="F84" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
@@ -19657,16 +19665,16 @@
     </row>
     <row r="85" customHeight="1" spans="1:26">
       <c r="A85" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B85" s="5"/>
       <c r="C85" s="5"/>
       <c r="D85" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E85" s="5"/>
       <c r="F85" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G85" s="4"/>
       <c r="H85" s="4"/>
@@ -19691,16 +19699,16 @@
     </row>
     <row r="86" customHeight="1" spans="1:26">
       <c r="A86" s="6" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="6"/>
       <c r="D86" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E86" s="6"/>
       <c r="F86" s="6" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
@@ -19725,16 +19733,16 @@
     </row>
     <row r="87" customHeight="1" spans="1:26">
       <c r="A87" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E87" s="2"/>
       <c r="F87" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G87" s="4"/>
       <c r="H87" s="4"/>
@@ -19759,16 +19767,16 @@
     </row>
     <row r="88" customHeight="1" spans="1:26">
       <c r="A88" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B88" s="5"/>
       <c r="C88" s="5"/>
       <c r="D88" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E88" s="5"/>
       <c r="F88" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
@@ -19793,16 +19801,16 @@
     </row>
     <row r="89" customHeight="1" spans="1:26">
       <c r="A89" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B89" s="5"/>
       <c r="C89" s="5"/>
       <c r="D89" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E89" s="5"/>
       <c r="F89" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
@@ -19827,16 +19835,16 @@
     </row>
     <row r="90" customHeight="1" spans="1:26">
       <c r="A90" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B90" s="5"/>
       <c r="C90" s="5"/>
       <c r="D90" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E90" s="5"/>
       <c r="F90" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="4"/>
@@ -19861,16 +19869,16 @@
     </row>
     <row r="91" customHeight="1" spans="1:26">
       <c r="A91" s="6" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B91" s="6"/>
       <c r="C91" s="6"/>
       <c r="D91" s="6" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E91" s="6"/>
       <c r="F91" s="6" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
@@ -19895,16 +19903,16 @@
     </row>
     <row r="92" customHeight="1" spans="1:26">
       <c r="A92" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E92" s="2"/>
       <c r="F92" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
@@ -19929,16 +19937,16 @@
     </row>
     <row r="93" customHeight="1" spans="1:26">
       <c r="A93" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B93" s="5"/>
       <c r="C93" s="5"/>
       <c r="D93" s="5" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E93" s="5"/>
       <c r="F93" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
@@ -19963,16 +19971,16 @@
     </row>
     <row r="94" customHeight="1" spans="1:26">
       <c r="A94" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B94" s="5"/>
       <c r="C94" s="5"/>
       <c r="D94" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E94" s="5"/>
       <c r="F94" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
@@ -19997,16 +20005,16 @@
     </row>
     <row r="95" customHeight="1" spans="1:26">
       <c r="A95" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B95" s="5"/>
       <c r="C95" s="5"/>
       <c r="D95" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G95" s="4"/>
       <c r="H95" s="4"/>
@@ -20031,16 +20039,16 @@
     </row>
     <row r="96" customHeight="1" spans="1:26">
       <c r="A96" s="6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B96" s="6"/>
       <c r="C96" s="6"/>
       <c r="D96" s="6" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E96" s="6"/>
       <c r="F96" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
@@ -20065,16 +20073,16 @@
     </row>
     <row r="97" customHeight="1" spans="1:26">
       <c r="A97" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E97" s="2"/>
       <c r="F97" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
@@ -20099,16 +20107,16 @@
     </row>
     <row r="98" customHeight="1" spans="1:26">
       <c r="A98" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="5"/>
       <c r="D98" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
@@ -20133,16 +20141,16 @@
     </row>
     <row r="99" customHeight="1" spans="1:26">
       <c r="A99" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B99" s="5"/>
       <c r="C99" s="5"/>
       <c r="D99" s="5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E99" s="5"/>
       <c r="F99" s="5" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
@@ -20167,16 +20175,16 @@
     </row>
     <row r="100" customHeight="1" spans="1:26">
       <c r="A100" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B100" s="5"/>
       <c r="C100" s="5"/>
       <c r="D100" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E100" s="5"/>
       <c r="F100" s="5" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G100" s="4"/>
       <c r="H100" s="4"/>
@@ -20201,16 +20209,16 @@
     </row>
     <row r="101" customHeight="1" spans="1:26">
       <c r="A101" s="6" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="6"/>
       <c r="D101" s="6" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E101" s="6"/>
       <c r="F101" s="6" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G101" s="4"/>
       <c r="H101" s="4"/>
@@ -20235,16 +20243,16 @@
     </row>
     <row r="102" customHeight="1" spans="1:26">
       <c r="A102" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
       <c r="D102" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E102" s="2"/>
       <c r="F102" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G102" s="4"/>
       <c r="H102" s="4"/>
@@ -20269,16 +20277,16 @@
     </row>
     <row r="103" customHeight="1" spans="1:26">
       <c r="A103" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B103" s="5"/>
       <c r="C103" s="5"/>
       <c r="D103" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E103" s="5"/>
       <c r="F103" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
@@ -20303,16 +20311,16 @@
     </row>
     <row r="104" customHeight="1" spans="1:26">
       <c r="A104" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B104" s="5"/>
       <c r="C104" s="5"/>
       <c r="D104" s="5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E104" s="5"/>
       <c r="F104" s="5" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="4"/>
@@ -20337,16 +20345,16 @@
     </row>
     <row r="105" customHeight="1" spans="1:26">
       <c r="A105" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B105" s="5"/>
       <c r="C105" s="5"/>
       <c r="D105" s="5" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E105" s="5"/>
       <c r="F105" s="5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
@@ -20371,16 +20379,16 @@
     </row>
     <row r="106" customHeight="1" spans="1:26">
       <c r="A106" s="6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="6"/>
       <c r="D106" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E106" s="6"/>
       <c r="F106" s="6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G106" s="4"/>
       <c r="H106" s="4"/>
@@ -20405,16 +20413,16 @@
     </row>
     <row r="107" customHeight="1" spans="1:26">
       <c r="A107" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
       <c r="D107" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E107" s="2"/>
       <c r="F107" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G107" s="4"/>
       <c r="H107" s="4"/>
@@ -20439,16 +20447,16 @@
     </row>
     <row r="108" customHeight="1" spans="1:26">
       <c r="A108" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B108" s="5"/>
       <c r="C108" s="5"/>
       <c r="D108" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E108" s="5"/>
       <c r="F108" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G108" s="4"/>
       <c r="H108" s="4"/>
@@ -20473,16 +20481,16 @@
     </row>
     <row r="109" customHeight="1" spans="1:26">
       <c r="A109" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B109" s="5"/>
       <c r="C109" s="5"/>
       <c r="D109" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E109" s="5"/>
       <c r="F109" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G109" s="4"/>
       <c r="H109" s="4"/>
@@ -20507,16 +20515,16 @@
     </row>
     <row r="110" customHeight="1" spans="1:26">
       <c r="A110" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B110" s="5"/>
       <c r="C110" s="5"/>
       <c r="D110" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E110" s="5"/>
       <c r="F110" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G110" s="4"/>
       <c r="H110" s="4"/>
@@ -20541,16 +20549,16 @@
     </row>
     <row r="111" customHeight="1" spans="1:26">
       <c r="A111" s="6" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="6"/>
       <c r="D111" s="6" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E111" s="6"/>
       <c r="F111" s="6" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G111" s="4"/>
       <c r="H111" s="4"/>
@@ -20575,16 +20583,16 @@
     </row>
     <row r="112" customHeight="1" spans="1:26">
       <c r="A112" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
       <c r="D112" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E112" s="2"/>
       <c r="F112" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112" s="4"/>
@@ -20609,16 +20617,16 @@
     </row>
     <row r="113" customHeight="1" spans="1:26">
       <c r="A113" s="5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B113" s="5"/>
       <c r="C113" s="5"/>
       <c r="D113" s="5" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E113" s="5"/>
       <c r="F113" s="5" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
@@ -20643,16 +20651,16 @@
     </row>
     <row r="114" customHeight="1" spans="1:26">
       <c r="A114" s="5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B114" s="5"/>
       <c r="C114" s="5"/>
       <c r="D114" s="5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E114" s="5"/>
       <c r="F114" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G114" s="4"/>
       <c r="H114" s="4"/>
@@ -20677,16 +20685,16 @@
     </row>
     <row r="115" customHeight="1" spans="1:26">
       <c r="A115" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B115" s="5"/>
       <c r="C115" s="5"/>
       <c r="D115" s="5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E115" s="5"/>
       <c r="F115" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
@@ -20711,16 +20719,16 @@
     </row>
     <row r="116" customHeight="1" spans="1:26">
       <c r="A116" s="6" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B116" s="6"/>
       <c r="C116" s="6"/>
       <c r="D116" s="6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E116" s="6"/>
       <c r="F116" s="6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G116" s="4"/>
       <c r="H116" s="4"/>
@@ -20745,16 +20753,16 @@
     </row>
     <row r="117" customHeight="1" spans="1:26">
       <c r="A117" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
       <c r="D117" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E117" s="2"/>
       <c r="F117" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="G117" s="4"/>
       <c r="H117" s="4"/>
@@ -20779,16 +20787,16 @@
     </row>
     <row r="118" customHeight="1" spans="1:26">
       <c r="A118" s="5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B118" s="5"/>
       <c r="C118" s="5"/>
       <c r="D118" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E118" s="5"/>
       <c r="F118" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G118" s="4"/>
       <c r="H118" s="4"/>
@@ -20813,16 +20821,16 @@
     </row>
     <row r="119" customHeight="1" spans="1:26">
       <c r="A119" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B119" s="5"/>
       <c r="C119" s="5"/>
       <c r="D119" s="5" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E119" s="5"/>
       <c r="F119" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G119" s="4"/>
       <c r="H119" s="4"/>
@@ -20847,16 +20855,16 @@
     </row>
     <row r="120" customHeight="1" spans="1:26">
       <c r="A120" s="5" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B120" s="5"/>
       <c r="C120" s="5"/>
       <c r="D120" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E120" s="5"/>
       <c r="F120" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G120" s="4"/>
       <c r="H120" s="4"/>
@@ -20881,16 +20889,16 @@
     </row>
     <row r="121" customHeight="1" spans="1:26">
       <c r="A121" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B121" s="6"/>
       <c r="C121" s="6"/>
       <c r="D121" s="6" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E121" s="6"/>
       <c r="F121" s="6" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G121" s="4"/>
       <c r="H121" s="4"/>
@@ -20915,16 +20923,16 @@
     </row>
     <row r="122" customHeight="1" spans="1:26">
       <c r="A122" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
       <c r="D122" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E122" s="2"/>
       <c r="F122" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
@@ -20949,16 +20957,16 @@
     </row>
     <row r="123" customHeight="1" spans="1:26">
       <c r="A123" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B123" s="5"/>
       <c r="C123" s="5"/>
       <c r="D123" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="5" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G123" s="4"/>
       <c r="H123" s="4"/>
@@ -20983,16 +20991,16 @@
     </row>
     <row r="124" customHeight="1" spans="1:26">
       <c r="A124" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B124" s="5"/>
       <c r="C124" s="5"/>
       <c r="D124" s="5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="G124" s="4"/>
       <c r="H124" s="4"/>
@@ -21017,16 +21025,16 @@
     </row>
     <row r="125" customHeight="1" spans="1:26">
       <c r="A125" s="5" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
       <c r="D125" s="5" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="E125" s="5"/>
       <c r="F125" s="5" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="G125" s="4"/>
       <c r="H125" s="4"/>
@@ -21051,16 +21059,16 @@
     </row>
     <row r="126" customHeight="1" spans="1:26">
       <c r="A126" s="6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B126" s="6"/>
       <c r="C126" s="6"/>
       <c r="D126" s="6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E126" s="6"/>
       <c r="F126" s="6" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G126" s="4"/>
       <c r="H126" s="4"/>
@@ -21085,16 +21093,16 @@
     </row>
     <row r="127" customHeight="1" spans="1:26">
       <c r="A127" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
       <c r="D127" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="E127" s="2"/>
       <c r="F127" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
@@ -21119,16 +21127,16 @@
     </row>
     <row r="128" customHeight="1" spans="1:26">
       <c r="A128" s="5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
       <c r="D128" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G128" s="4"/>
       <c r="H128" s="4"/>
@@ -21153,16 +21161,16 @@
     </row>
     <row r="129" customHeight="1" spans="1:26">
       <c r="A129" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
       <c r="D129" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E129" s="5"/>
       <c r="F129" s="5" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="G129" s="4"/>
       <c r="H129" s="4"/>
@@ -21187,16 +21195,16 @@
     </row>
     <row r="130" customHeight="1" spans="1:26">
       <c r="A130" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
       <c r="D130" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E130" s="5"/>
       <c r="F130" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G130" s="4"/>
       <c r="H130" s="4"/>
@@ -21221,16 +21229,16 @@
     </row>
     <row r="131" customHeight="1" spans="1:26">
       <c r="A131" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B131" s="6"/>
       <c r="C131" s="6"/>
       <c r="D131" s="6" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E131" s="6"/>
       <c r="F131" s="6" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="G131" s="4"/>
       <c r="H131" s="4"/>
@@ -21255,16 +21263,16 @@
     </row>
     <row r="132" customHeight="1" spans="1:26">
       <c r="A132" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
       <c r="D132" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E132" s="2"/>
       <c r="F132" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G132" s="4"/>
       <c r="H132" s="4"/>
@@ -21289,16 +21297,16 @@
     </row>
     <row r="133" customHeight="1" spans="1:26">
       <c r="A133" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
       <c r="D133" s="5" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="G133" s="4"/>
       <c r="H133" s="4"/>
@@ -21323,16 +21331,16 @@
     </row>
     <row r="134" customHeight="1" spans="1:26">
       <c r="A134" s="5" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
       <c r="D134" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E134" s="5"/>
       <c r="F134" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="G134" s="4"/>
       <c r="H134" s="4"/>
@@ -21357,16 +21365,16 @@
     </row>
     <row r="135" customHeight="1" spans="1:26">
       <c r="A135" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
       <c r="D135" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G135" s="4"/>
       <c r="H135" s="4"/>
@@ -21391,16 +21399,16 @@
     </row>
     <row r="136" customHeight="1" spans="1:26">
       <c r="A136" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B136" s="6"/>
       <c r="C136" s="6"/>
       <c r="D136" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E136" s="6"/>
       <c r="F136" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G136" s="4"/>
       <c r="H136" s="4"/>
@@ -21425,16 +21433,16 @@
     </row>
     <row r="137" customHeight="1" spans="1:26">
       <c r="A137" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
       <c r="D137" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E137" s="2"/>
       <c r="F137" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G137" s="4"/>
       <c r="H137" s="4"/>
@@ -21459,16 +21467,16 @@
     </row>
     <row r="138" customHeight="1" spans="1:26">
       <c r="A138" s="5" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B138" s="5"/>
       <c r="C138" s="5"/>
       <c r="D138" s="5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G138" s="4"/>
       <c r="H138" s="4"/>
@@ -21493,16 +21501,16 @@
     </row>
     <row r="139" customHeight="1" spans="1:26">
       <c r="A139" s="5" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B139" s="5"/>
       <c r="C139" s="5"/>
       <c r="D139" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="G139" s="4"/>
       <c r="H139" s="4"/>
@@ -21527,16 +21535,16 @@
     </row>
     <row r="140" customHeight="1" spans="1:26">
       <c r="A140" s="5" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B140" s="5"/>
       <c r="C140" s="5"/>
       <c r="D140" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E140" s="5"/>
       <c r="F140" s="5" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G140" s="4"/>
       <c r="H140" s="4"/>
@@ -21561,16 +21569,16 @@
     </row>
     <row r="141" customHeight="1" spans="1:26">
       <c r="A141" s="6" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B141" s="6"/>
       <c r="C141" s="6"/>
       <c r="D141" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="E141" s="6"/>
       <c r="F141" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="G141" s="4"/>
       <c r="H141" s="4"/>
@@ -21595,16 +21603,16 @@
     </row>
     <row r="142" customHeight="1" spans="1:26">
       <c r="A142" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
       <c r="D142" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="E142" s="2"/>
       <c r="F142" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G142" s="4"/>
       <c r="H142" s="4"/>
@@ -21629,16 +21637,16 @@
     </row>
     <row r="143" customHeight="1" spans="1:26">
       <c r="A143" s="5" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
       <c r="D143" s="5" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E143" s="5"/>
       <c r="F143" s="5" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="G143" s="4"/>
       <c r="H143" s="4"/>
@@ -21663,16 +21671,16 @@
     </row>
     <row r="144" customHeight="1" spans="1:26">
       <c r="A144" s="5" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B144" s="5"/>
       <c r="C144" s="5"/>
       <c r="D144" s="5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E144" s="5"/>
       <c r="F144" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G144" s="4"/>
       <c r="H144" s="4"/>
@@ -21697,16 +21705,16 @@
     </row>
     <row r="145" customHeight="1" spans="1:26">
       <c r="A145" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
       <c r="D145" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="E145" s="5"/>
       <c r="F145" s="5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="G145" s="4"/>
       <c r="H145" s="4"/>
@@ -21731,16 +21739,16 @@
     </row>
     <row r="146" customHeight="1" spans="1:26">
       <c r="A146" s="6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="6"/>
       <c r="D146" s="6" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E146" s="6"/>
       <c r="F146" s="6" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="G146" s="4"/>
       <c r="H146" s="4"/>
@@ -21765,16 +21773,16 @@
     </row>
     <row r="147" customHeight="1" spans="1:26">
       <c r="A147" s="2" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
       <c r="D147" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E147" s="2"/>
       <c r="F147" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="G147" s="4"/>
       <c r="H147" s="4"/>
@@ -21799,16 +21807,16 @@
     </row>
     <row r="148" customHeight="1" spans="1:26">
       <c r="A148" s="5" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
       <c r="D148" s="5" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E148" s="5"/>
       <c r="F148" s="5" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G148" s="4"/>
       <c r="H148" s="4"/>
@@ -21833,16 +21841,16 @@
     </row>
     <row r="149" customHeight="1" spans="1:26">
       <c r="A149" s="5" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
       <c r="D149" s="5" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="E149" s="5"/>
       <c r="F149" s="5" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G149" s="4"/>
       <c r="H149" s="4"/>
@@ -21867,16 +21875,16 @@
     </row>
     <row r="150" customHeight="1" spans="1:26">
       <c r="A150" s="5" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
       <c r="D150" s="5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E150" s="5"/>
       <c r="F150" s="5" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="G150" s="4"/>
       <c r="H150" s="4"/>
@@ -21901,16 +21909,16 @@
     </row>
     <row r="151" customHeight="1" spans="1:26">
       <c r="A151" s="6" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B151" s="6"/>
       <c r="C151" s="6"/>
       <c r="D151" s="6" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E151" s="6"/>
       <c r="F151" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="G151" s="4"/>
       <c r="H151" s="4"/>
@@ -21935,16 +21943,16 @@
     </row>
     <row r="152" customHeight="1" spans="1:26">
       <c r="A152" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
       <c r="D152" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E152" s="2"/>
       <c r="F152" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G152" s="4"/>
       <c r="H152" s="4"/>
@@ -21969,16 +21977,16 @@
     </row>
     <row r="153" customHeight="1" spans="1:26">
       <c r="A153" s="5" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
       <c r="D153" s="5" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E153" s="5"/>
       <c r="F153" s="5" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="G153" s="4"/>
       <c r="H153" s="4"/>
@@ -22003,16 +22011,16 @@
     </row>
     <row r="154" customHeight="1" spans="1:26">
       <c r="A154" s="5" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
       <c r="D154" s="5" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E154" s="5"/>
       <c r="F154" s="5" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="G154" s="4"/>
       <c r="H154" s="4"/>
@@ -22037,16 +22045,16 @@
     </row>
     <row r="155" customHeight="1" spans="1:26">
       <c r="A155" s="5" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B155" s="5"/>
       <c r="C155" s="5"/>
       <c r="D155" s="5" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E155" s="5"/>
       <c r="F155" s="5" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G155" s="4"/>
       <c r="H155" s="4"/>
@@ -22071,16 +22079,16 @@
     </row>
     <row r="156" customHeight="1" spans="1:26">
       <c r="A156" s="6" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B156" s="6"/>
       <c r="C156" s="6"/>
       <c r="D156" s="6" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E156" s="6"/>
       <c r="F156" s="6" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="G156" s="4"/>
       <c r="H156" s="4"/>
@@ -22105,16 +22113,16 @@
     </row>
     <row r="157" customHeight="1" spans="1:26">
       <c r="A157" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
       <c r="D157" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E157" s="2"/>
       <c r="F157" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="G157" s="4"/>
       <c r="H157" s="4"/>
@@ -22139,16 +22147,16 @@
     </row>
     <row r="158" customHeight="1" spans="1:26">
       <c r="A158" s="5" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B158" s="5"/>
       <c r="C158" s="5"/>
       <c r="D158" s="5" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="E158" s="5"/>
       <c r="F158" s="5" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G158" s="4"/>
       <c r="H158" s="4"/>
@@ -22173,16 +22181,16 @@
     </row>
     <row r="159" customHeight="1" spans="1:26">
       <c r="A159" s="5" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B159" s="5"/>
       <c r="C159" s="5"/>
       <c r="D159" s="5" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E159" s="5"/>
       <c r="F159" s="5" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="G159" s="4"/>
       <c r="H159" s="4"/>
@@ -22207,16 +22215,16 @@
     </row>
     <row r="160" customHeight="1" spans="1:26">
       <c r="A160" s="5" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B160" s="5"/>
       <c r="C160" s="5"/>
       <c r="D160" s="5" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="E160" s="5"/>
       <c r="F160" s="5" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="G160" s="4"/>
       <c r="H160" s="4"/>
@@ -22241,16 +22249,16 @@
     </row>
     <row r="161" customHeight="1" spans="1:26">
       <c r="A161" s="6" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B161" s="6"/>
       <c r="C161" s="6"/>
       <c r="D161" s="6" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="E161" s="6"/>
       <c r="F161" s="6" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G161" s="4"/>
       <c r="H161" s="4"/>
@@ -22275,16 +22283,16 @@
     </row>
     <row r="162" customHeight="1" spans="1:26">
       <c r="A162" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
       <c r="D162" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="E162" s="2"/>
       <c r="F162" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="G162" s="4"/>
       <c r="H162" s="4"/>
@@ -22309,16 +22317,16 @@
     </row>
     <row r="163" customHeight="1" spans="1:26">
       <c r="A163" s="5" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B163" s="5"/>
       <c r="C163" s="5"/>
       <c r="D163" s="5" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="E163" s="5"/>
       <c r="F163" s="5" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="G163" s="4"/>
       <c r="H163" s="4"/>
@@ -22343,16 +22351,16 @@
     </row>
     <row r="164" customHeight="1" spans="1:26">
       <c r="A164" s="5" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B164" s="5"/>
       <c r="C164" s="5"/>
       <c r="D164" s="5" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="E164" s="5"/>
       <c r="F164" s="5" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="G164" s="4"/>
       <c r="H164" s="4"/>
@@ -22377,16 +22385,16 @@
     </row>
     <row r="165" customHeight="1" spans="1:26">
       <c r="A165" s="5" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B165" s="5"/>
       <c r="C165" s="5"/>
       <c r="D165" s="5" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="E165" s="5"/>
       <c r="F165" s="5" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="G165" s="4"/>
       <c r="H165" s="4"/>
@@ -22411,16 +22419,16 @@
     </row>
     <row r="166" customHeight="1" spans="1:26">
       <c r="A166" s="6" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B166" s="6"/>
       <c r="C166" s="6"/>
       <c r="D166" s="6" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E166" s="6"/>
       <c r="F166" s="6" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="G166" s="4"/>
       <c r="H166" s="4"/>
@@ -22445,16 +22453,16 @@
     </row>
     <row r="167" customHeight="1" spans="1:26">
       <c r="A167" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
       <c r="D167" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E167" s="2"/>
       <c r="F167" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="G167" s="4"/>
       <c r="H167" s="4"/>
@@ -22479,16 +22487,16 @@
     </row>
     <row r="168" customHeight="1" spans="1:26">
       <c r="A168" s="5" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B168" s="5"/>
       <c r="C168" s="5"/>
       <c r="D168" s="5" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E168" s="5"/>
       <c r="F168" s="5" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="G168" s="4"/>
       <c r="H168" s="4"/>
@@ -22513,16 +22521,16 @@
     </row>
     <row r="169" customHeight="1" spans="1:26">
       <c r="A169" s="5" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B169" s="5"/>
       <c r="C169" s="5"/>
       <c r="D169" s="5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="E169" s="5"/>
       <c r="F169" s="5" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="G169" s="4"/>
       <c r="H169" s="4"/>
@@ -22547,16 +22555,16 @@
     </row>
     <row r="170" customHeight="1" spans="1:26">
       <c r="A170" s="5" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B170" s="5"/>
       <c r="C170" s="5"/>
       <c r="D170" s="5" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E170" s="5"/>
       <c r="F170" s="5" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G170" s="4"/>
       <c r="H170" s="4"/>
@@ -22581,16 +22589,16 @@
     </row>
     <row r="171" customHeight="1" spans="1:26">
       <c r="A171" s="6" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B171" s="6"/>
       <c r="C171" s="6"/>
       <c r="D171" s="6" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E171" s="6"/>
       <c r="F171" s="6" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G171" s="4"/>
       <c r="H171" s="4"/>
@@ -22615,16 +22623,16 @@
     </row>
     <row r="172" customHeight="1" spans="1:26">
       <c r="A172" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
       <c r="D172" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E172" s="2"/>
       <c r="F172" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="G172" s="4"/>
       <c r="H172" s="4"/>
@@ -22649,16 +22657,16 @@
     </row>
     <row r="173" customHeight="1" spans="1:26">
       <c r="A173" s="5" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B173" s="5"/>
       <c r="C173" s="5"/>
       <c r="D173" s="5" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E173" s="5"/>
       <c r="F173" s="5" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G173" s="4"/>
       <c r="H173" s="4"/>
@@ -22683,16 +22691,16 @@
     </row>
     <row r="174" customHeight="1" spans="1:26">
       <c r="A174" s="5" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B174" s="5"/>
       <c r="C174" s="5"/>
       <c r="D174" s="5" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E174" s="5"/>
       <c r="F174" s="5" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="G174" s="4"/>
       <c r="H174" s="4"/>
@@ -22717,16 +22725,16 @@
     </row>
     <row r="175" customHeight="1" spans="1:26">
       <c r="A175" s="5" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B175" s="5"/>
       <c r="C175" s="5"/>
       <c r="D175" s="5" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="E175" s="5"/>
       <c r="F175" s="5" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="G175" s="4"/>
       <c r="H175" s="4"/>
@@ -22751,16 +22759,16 @@
     </row>
     <row r="176" customHeight="1" spans="1:26">
       <c r="A176" s="6" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B176" s="6"/>
       <c r="C176" s="6"/>
       <c r="D176" s="6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E176" s="6"/>
       <c r="F176" s="6" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="G176" s="4"/>
       <c r="H176" s="4"/>
@@ -22785,16 +22793,16 @@
     </row>
     <row r="177" customHeight="1" spans="1:26">
       <c r="A177" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
       <c r="D177" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="E177" s="2"/>
       <c r="F177" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="G177" s="4"/>
       <c r="H177" s="4"/>
@@ -22819,16 +22827,16 @@
     </row>
     <row r="178" customHeight="1" spans="1:26">
       <c r="A178" s="5" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B178" s="5"/>
       <c r="C178" s="5"/>
       <c r="D178" s="5" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="E178" s="5"/>
       <c r="F178" s="5" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="G178" s="4"/>
       <c r="H178" s="4"/>
@@ -22853,16 +22861,16 @@
     </row>
     <row r="179" customHeight="1" spans="1:26">
       <c r="A179" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B179" s="5"/>
       <c r="C179" s="5"/>
       <c r="D179" s="5" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E179" s="5"/>
       <c r="F179" s="5" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="G179" s="4"/>
       <c r="H179" s="4"/>
@@ -22887,16 +22895,16 @@
     </row>
     <row r="180" customHeight="1" spans="1:26">
       <c r="A180" s="5" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B180" s="5"/>
       <c r="C180" s="5"/>
       <c r="D180" s="5" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E180" s="5"/>
       <c r="F180" s="5" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="G180" s="4"/>
       <c r="H180" s="4"/>
@@ -22921,16 +22929,16 @@
     </row>
     <row r="181" customHeight="1" spans="1:26">
       <c r="A181" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B181" s="6"/>
       <c r="C181" s="6"/>
       <c r="D181" s="6" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="E181" s="6"/>
       <c r="F181" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="G181" s="4"/>
       <c r="H181" s="4"/>
@@ -22955,16 +22963,16 @@
     </row>
     <row r="182" customHeight="1" spans="1:26">
       <c r="A182" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="E182" s="2"/>
       <c r="F182" s="2" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="G182" s="4"/>
       <c r="H182" s="4"/>
@@ -22989,16 +22997,16 @@
     </row>
     <row r="183" customHeight="1" spans="1:26">
       <c r="A183" s="5" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B183" s="5"/>
       <c r="C183" s="5"/>
       <c r="D183" s="5" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="E183" s="5"/>
       <c r="F183" s="5" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="G183" s="4"/>
       <c r="H183" s="4"/>
@@ -23023,16 +23031,16 @@
     </row>
     <row r="184" customHeight="1" spans="1:26">
       <c r="A184" s="5" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B184" s="5"/>
       <c r="C184" s="5"/>
       <c r="D184" s="5" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E184" s="5"/>
       <c r="F184" s="5" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="G184" s="4"/>
       <c r="H184" s="4"/>
@@ -23057,16 +23065,16 @@
     </row>
     <row r="185" customHeight="1" spans="1:26">
       <c r="A185" s="5" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B185" s="5"/>
       <c r="C185" s="5"/>
       <c r="D185" s="5" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="E185" s="5"/>
       <c r="F185" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="G185" s="4"/>
       <c r="H185" s="4"/>
@@ -23091,16 +23099,16 @@
     </row>
     <row r="186" customHeight="1" spans="1:26">
       <c r="A186" s="6" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B186" s="6"/>
       <c r="C186" s="6"/>
       <c r="D186" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="E186" s="6"/>
       <c r="F186" s="6" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="G186" s="4"/>
       <c r="H186" s="4"/>
@@ -23125,16 +23133,16 @@
     </row>
     <row r="187" customHeight="1" spans="1:26">
       <c r="A187" s="2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
       <c r="D187" s="2" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E187" s="2"/>
       <c r="F187" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="G187" s="4"/>
       <c r="H187" s="4"/>
@@ -23159,16 +23167,16 @@
     </row>
     <row r="188" customHeight="1" spans="1:26">
       <c r="A188" s="5" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B188" s="5"/>
       <c r="C188" s="5"/>
       <c r="D188" s="5" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="E188" s="5"/>
       <c r="F188" s="5" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="G188" s="4"/>
       <c r="H188" s="4"/>
@@ -23193,16 +23201,16 @@
     </row>
     <row r="189" customHeight="1" spans="1:26">
       <c r="A189" s="5" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B189" s="5"/>
       <c r="C189" s="5"/>
       <c r="D189" s="5" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="E189" s="5"/>
       <c r="F189" s="5" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="G189" s="4"/>
       <c r="H189" s="4"/>
@@ -23227,16 +23235,16 @@
     </row>
     <row r="190" customHeight="1" spans="1:26">
       <c r="A190" s="5" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B190" s="5"/>
       <c r="C190" s="5"/>
       <c r="D190" s="5" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E190" s="5"/>
       <c r="F190" s="5" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="G190" s="4"/>
       <c r="H190" s="4"/>
@@ -23261,16 +23269,16 @@
     </row>
     <row r="191" customHeight="1" spans="1:26">
       <c r="A191" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B191" s="6"/>
       <c r="C191" s="6"/>
       <c r="D191" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E191" s="6"/>
       <c r="F191" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G191" s="4"/>
       <c r="H191" s="4"/>
@@ -23295,16 +23303,16 @@
     </row>
     <row r="192" customHeight="1" spans="1:26">
       <c r="A192" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
       <c r="D192" s="2" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="E192" s="2"/>
       <c r="F192" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="G192" s="4"/>
       <c r="H192" s="4"/>
@@ -23329,16 +23337,16 @@
     </row>
     <row r="193" customHeight="1" spans="1:26">
       <c r="A193" s="5" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B193" s="5"/>
       <c r="C193" s="5"/>
       <c r="D193" s="5" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E193" s="5"/>
       <c r="F193" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="G193" s="4"/>
       <c r="H193" s="4"/>
@@ -23363,16 +23371,16 @@
     </row>
     <row r="194" customHeight="1" spans="1:26">
       <c r="A194" s="5" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B194" s="5"/>
       <c r="C194" s="5"/>
       <c r="D194" s="5" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E194" s="5"/>
       <c r="F194" s="5" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="G194" s="4"/>
       <c r="H194" s="4"/>
@@ -23397,16 +23405,16 @@
     </row>
     <row r="195" customHeight="1" spans="1:26">
       <c r="A195" s="5" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B195" s="5"/>
       <c r="C195" s="5"/>
       <c r="D195" s="5" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E195" s="5"/>
       <c r="F195" s="5" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G195" s="4"/>
       <c r="H195" s="4"/>
@@ -23431,16 +23439,16 @@
     </row>
     <row r="196" customHeight="1" spans="1:26">
       <c r="A196" s="6" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B196" s="6"/>
       <c r="C196" s="6"/>
       <c r="D196" s="6" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="E196" s="6"/>
       <c r="F196" s="6" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="G196" s="4"/>
       <c r="H196" s="4"/>
@@ -23465,16 +23473,16 @@
     </row>
     <row r="197" customHeight="1" spans="1:26">
       <c r="A197" s="2" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
       <c r="D197" s="2" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="E197" s="2"/>
       <c r="F197" s="2" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="G197" s="4"/>
       <c r="H197" s="4"/>
@@ -23499,16 +23507,16 @@
     </row>
     <row r="198" customHeight="1" spans="1:26">
       <c r="A198" s="5" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B198" s="5"/>
       <c r="C198" s="5"/>
       <c r="D198" s="5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="E198" s="5"/>
       <c r="F198" s="5" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="G198" s="4"/>
       <c r="H198" s="4"/>
@@ -23533,16 +23541,16 @@
     </row>
     <row r="199" customHeight="1" spans="1:26">
       <c r="A199" s="5" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B199" s="5"/>
       <c r="C199" s="5"/>
       <c r="D199" s="5" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E199" s="5"/>
       <c r="F199" s="5" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="G199" s="4"/>
       <c r="H199" s="4"/>
@@ -23567,16 +23575,16 @@
     </row>
     <row r="200" customHeight="1" spans="1:26">
       <c r="A200" s="5" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B200" s="5"/>
       <c r="C200" s="5"/>
       <c r="D200" s="5" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="E200" s="5"/>
       <c r="F200" s="5" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="G200" s="4"/>
       <c r="H200" s="4"/>
@@ -23601,16 +23609,16 @@
     </row>
     <row r="201" customHeight="1" spans="1:26">
       <c r="A201" s="6" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B201" s="6"/>
       <c r="C201" s="6"/>
       <c r="D201" s="6" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E201" s="6"/>
       <c r="F201" s="7" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="G201" s="4"/>
       <c r="H201" s="4"/>

</xml_diff>